<commit_message>
Updates for enhacements are in progress
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1E70CE-48A8-4AA8-BCF3-57A0E313AB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
   <si>
     <t>Transaction</t>
   </si>
@@ -32,9 +32,6 @@
   </si>
   <si>
     <t>Step3</t>
-  </si>
-  <si>
-    <t>ZMG002_01</t>
   </si>
   <si>
     <t>variante</t>
@@ -938,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -955,29 +952,29 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -985,24 +982,24 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>6</v>
+      <c r="D4" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1010,18 +1007,18 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1029,10 +1026,13 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
         <v>5</v>
       </c>
-      <c r="C8" t="s">
-        <v>6</v>
+      <c r="D8" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1040,13 +1040,10 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1054,32 +1051,21 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
         <v>5</v>
       </c>
-      <c r="C10" t="s">
-        <v>6</v>
+      <c r="E10" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
       <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates were completed, success execution was completed
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1E70CE-48A8-4AA8-BCF3-57A0E313AB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
   <si>
     <t>Transaction</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>Step3</t>
+  </si>
+  <si>
+    <t>ZMG002_01</t>
   </si>
   <si>
     <t>variante</t>
@@ -935,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -952,29 +955,29 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -982,24 +985,24 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1007,18 +1010,18 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
         <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1026,13 +1029,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1040,10 +1040,13 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1051,21 +1054,32 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
         <v>5</v>
       </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update to remove empty rows before headers was completed.
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B87B7E26-03D8-4547-B2AE-0FC72D09FC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Transaction</t>
   </si>
@@ -34,31 +34,13 @@
     <t>Step3</t>
   </si>
   <si>
-    <t>ZMG002_01</t>
-  </si>
-  <si>
     <t>variante</t>
   </si>
   <si>
     <t>ejecutar</t>
   </si>
   <si>
-    <t>ZMM026</t>
-  </si>
-  <si>
-    <t>disposicion</t>
-  </si>
-  <si>
     <t>LX02</t>
-  </si>
-  <si>
-    <t>COHV</t>
-  </si>
-  <si>
-    <t>checks</t>
-  </si>
-  <si>
-    <t>ZCO017</t>
   </si>
   <si>
     <t>ZPP029_1</t>
@@ -67,31 +49,7 @@
     <t>BOM</t>
   </si>
   <si>
-    <t>MB52</t>
-  </si>
-  <si>
-    <t>ZSD053</t>
-  </si>
-  <si>
-    <t>LT23</t>
-  </si>
-  <si>
-    <t>VL06O</t>
-  </si>
-  <si>
-    <t>listas sal</t>
-  </si>
-  <si>
-    <t>vista posicion</t>
-  </si>
-  <si>
-    <t>ODM</t>
-  </si>
-  <si>
     <t>Step4</t>
-  </si>
-  <si>
-    <t>filtrar pedido</t>
   </si>
 </sst>
 </file>
@@ -581,8 +539,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -938,7 +897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -955,131 +914,26 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>